<commit_message>
nieuws opvragen werkt, poster en rapport/werkstuk ook af
</commit_message>
<xml_diff>
--- a/stage/Logblad_Stage.xlsx
+++ b/stage/Logblad_Stage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tbelm\Documenten\Graduaat-Programmeren\stage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DCFD3C9-DA9F-4DEC-BF49-3223FD328D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98BAD9D4-2266-4333-B288-680FB875E5A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{17B13AA9-2AFD-4646-A20A-7BB5FF3EC105}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="179">
   <si>
     <t>Logblad Stage</t>
   </si>
@@ -742,6 +742,22 @@
 om deze templates op een overzichtelijke en visueel aantrekkelijke manier weer te geven op het scherm.
 Daarna heb ik onze projectbrede Toolbar geïntegreerd, zodat gebruikers kunnen filteren op naam en sorteren op aanmaakdatum of laatste wijziging. Tot slot heb ik ervoor gezorgd dat wanneer je op een e-mailtemplate klikt, je wordt doorgestuurd naar de e-maileditor,
 waar je de template verder kunt bewerken.</t>
+  </si>
+  <si>
+    <t>EmailPage backend kopppelen met frontend</t>
+  </si>
+  <si>
+    <t>Vandaag was mijn laatste stagedag.
+Als afsluitende opdracht kreeg ik de taak om de previewpagina van de e-mails af te werken. Ik begon hier meteen aan en had deze vrij snel klaar. Daarna kreeg ik de kans om mijn volledige code nog eens grondig te testen en op verschillende plaatsen kleine verbeteringen door te voeren. Zo voegde ik bijvoorbeeld een veld toe om te tonen of een e-mailtemplate al gepubliceerd was of niet.
+Het was een zeer leerrijke stage, waarin ik veel verantwoordelijkheden kreeg en enorm veel heb bijgeleerd. Ik kijk met een positief gevoel terug op deze ervaring.</t>
+  </si>
+  <si>
+    <t>EmailPreview page aanmaken + laatste aanpassingen code</t>
+  </si>
+  <si>
+    <t>Vandaag werkte ik verder aan de e-mailpagina.
+ Vorige week heeft de backend developer de nodige API-calls voorzien voor het ophalen, aanmaken en updaten van e-mailtemplates. Vandaag heb ik deze integraties succesvol geïmplementeerd in mijn bestaande frontend-code en getest op correcte werking.
+Daarna ben ik gestart met mijn laatste opdracht: het opzetten van een nieuwe pagina waarop je een preview van de e-mails kunt bekijken in verschillende schermformaten, zoals desktop, laptop en mobiel. Dit is bedoeld om na te gaan hoe de e-mails zich gedragen op verschillende apparaten.</t>
   </si>
 </sst>
 </file>
@@ -1158,6 +1174,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1181,21 +1212,6 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1532,13 +1548,13 @@
     </row>
     <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="45"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="7"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1552,11 +1568,11 @@
       <c r="B4" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="41"/>
-      <c r="F4" s="42"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="34"/>
       <c r="G4" s="7"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1570,11 +1586,11 @@
       <c r="B6" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="41"/>
-      <c r="F6" s="42"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="34"/>
       <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1588,11 +1604,11 @@
       <c r="B8" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="41"/>
-      <c r="F8" s="42"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="34"/>
       <c r="G8" s="7"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1606,11 +1622,11 @@
       <c r="B10" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="41"/>
-      <c r="F10" s="42"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="34"/>
       <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1624,11 +1640,11 @@
       <c r="B12" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="41"/>
-      <c r="F12" s="42"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="34"/>
       <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -3283,28 +3299,28 @@
       </c>
     </row>
     <row r="104" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B104" s="37">
+      <c r="B104" s="42">
         <v>89</v>
       </c>
-      <c r="C104" s="39" t="s">
+      <c r="C104" s="44" t="s">
         <v>150</v>
       </c>
-      <c r="D104" s="33" t="s">
+      <c r="D104" s="38" t="s">
         <v>148</v>
       </c>
-      <c r="E104" s="33" t="s">
+      <c r="E104" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="F104" s="35" t="s">
+      <c r="F104" s="40" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="105" spans="2:6" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B105" s="38"/>
-      <c r="C105" s="40"/>
-      <c r="D105" s="34"/>
-      <c r="E105" s="34"/>
-      <c r="F105" s="36"/>
+      <c r="B105" s="43"/>
+      <c r="C105" s="45"/>
+      <c r="D105" s="39"/>
+      <c r="E105" s="39"/>
+      <c r="F105" s="41"/>
     </row>
     <row r="106" spans="2:6" ht="135" x14ac:dyDescent="0.25">
       <c r="B106" s="13">
@@ -3527,31 +3543,39 @@
         <v>174</v>
       </c>
     </row>
-    <row r="119" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:6" ht="120" x14ac:dyDescent="0.25">
       <c r="B119" s="13">
         <v>104</v>
       </c>
       <c r="C119" s="29">
         <v>45810</v>
       </c>
-      <c r="D119" s="14"/>
+      <c r="D119" s="14" t="s">
+        <v>175</v>
+      </c>
       <c r="E119" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="F119" s="14"/>
-    </row>
-    <row r="120" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F119" s="28" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="120" spans="2:6" ht="135" x14ac:dyDescent="0.25">
       <c r="B120" s="13">
         <v>105</v>
       </c>
       <c r="C120" s="29">
         <v>45811</v>
       </c>
-      <c r="D120" s="14"/>
+      <c r="D120" s="14" t="s">
+        <v>177</v>
+      </c>
       <c r="E120" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="F120" s="14"/>
+      <c r="F120" s="28" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="121" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B121" s="13">
@@ -3969,17 +3993,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="D104:D105"/>
+    <mergeCell ref="F104:F105"/>
+    <mergeCell ref="E104:E105"/>
+    <mergeCell ref="B104:B105"/>
+    <mergeCell ref="C104:C105"/>
     <mergeCell ref="D12:F12"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D104:D105"/>
-    <mergeCell ref="F104:F105"/>
-    <mergeCell ref="E104:E105"/>
-    <mergeCell ref="B104:B105"/>
-    <mergeCell ref="C104:C105"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3994,6 +4018,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E23CA4F9A7097943BB3661E90EAE6E4E" ma:contentTypeVersion="14" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="0d9e0f82b7cffe5fc1e74a09a28c1088">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="9bca8325-008a-4bac-8c6f-d19d7077bb5c" xmlns:ns4="9ad299d5-20ee-4f22-8259-94c3717e0ced" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fa769e857125b647229b5c2d99e2d252" ns3:_="" ns4:_="">
     <xsd:import namespace="9bca8325-008a-4bac-8c6f-d19d7077bb5c"/>
@@ -4222,15 +4255,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{875E8F8E-7746-48C0-A297-237F1A7749C7}">
   <ds:schemaRefs>
@@ -4241,6 +4265,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8784147-5A1F-4134-92F8-D5D0439B0E8D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{259DE696-BD32-4CBC-931A-5C4B7B33C4BA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4257,12 +4289,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8784147-5A1F-4134-92F8-D5D0439B0E8D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>